<commit_message>
Improve DeepSeek evidence collection
</commit_message>
<xml_diff>
--- a/questions.backup-before-more-questions.xlsx
+++ b/questions.backup-before-more-questions.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pan/Documents/思阳/geo-evidence-collector/yingdao_mvp/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pan/Documents/思阳/Automatic-screenshot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D001031-9268-3D43-8F62-E7B0E51573BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20621BF0-2647-DF45-87E3-622B31F346B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-2060" yWindow="-22000" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="56">
   <si>
     <t>id</t>
   </si>
@@ -38,21 +38,12 @@
     <t>status</t>
   </si>
   <si>
-    <t>Q001</t>
-  </si>
-  <si>
     <t>deepseek</t>
   </si>
   <si>
     <t>success</t>
   </si>
   <si>
-    <t>Q002</t>
-  </si>
-  <si>
-    <t>Q003</t>
-  </si>
-  <si>
     <t>Yingdao GEO Collector MVP</t>
   </si>
   <si>
@@ -182,27 +173,29 @@
     <t>Set status = success or failed with remark.</t>
   </si>
   <si>
-    <t>pending</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>推荐一下好用的厨具</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>推荐一下家用的柜式洗碗机</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>推荐几款隐藏式冰箱</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <t>Q031</t>
+  </si>
+  <si>
+    <t>推荐一下家用烘干机怎么选</t>
+  </si>
+  <si>
+    <t>Q032</t>
+  </si>
+  <si>
+    <t>推荐几款扫拖一体机器人</t>
+  </si>
+  <si>
+    <t>Q033</t>
+  </si>
+  <si>
+    <t>推荐一下适合家用的空气净化器</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -222,12 +215,6 @@
       <name val="FangSong"/>
       <family val="3"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Carlito"/>
     </font>
   </fonts>
   <fills count="3">
@@ -252,12 +239,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -269,12 +255,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="超链接" xfId="2" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -438,7 +422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J105"/>
+  <dimension ref="A1:I102"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
@@ -449,7 +433,7 @@
     <col min="9" max="9" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="20" customHeight="1">
+    <row r="1" spans="1:9" ht="20" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -470,71 +454,70 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
     </row>
-    <row r="2" spans="1:10" ht="94" customHeight="1">
+    <row r="2" spans="1:9" ht="26.75" customHeight="1">
       <c r="A2" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
-      <c r="J2" s="5"/>
-    </row>
-    <row r="3" spans="1:10" ht="89" customHeight="1">
+    </row>
+    <row r="3" spans="1:9" ht="26.75" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>53</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
     </row>
-    <row r="4" spans="1:10" ht="132" customHeight="1">
+    <row r="4" spans="1:9" ht="26.75" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>55</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
     </row>
-    <row r="5" spans="1:10" ht="20" customHeight="1">
+    <row r="5" spans="1:9" ht="20" customHeight="1">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -545,7 +528,7 @@
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
     </row>
-    <row r="6" spans="1:10" ht="20" customHeight="1">
+    <row r="6" spans="1:9" ht="20" customHeight="1">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -556,7 +539,7 @@
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
     </row>
-    <row r="7" spans="1:10" ht="20" customHeight="1">
+    <row r="7" spans="1:9" ht="20" customHeight="1">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -567,7 +550,7 @@
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
     </row>
-    <row r="8" spans="1:10" ht="20" customHeight="1">
+    <row r="8" spans="1:9" ht="20" customHeight="1">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -578,7 +561,7 @@
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
     </row>
-    <row r="9" spans="1:10" ht="20" customHeight="1">
+    <row r="9" spans="1:9" ht="20" customHeight="1">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -589,9 +572,9 @@
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
     </row>
-    <row r="10" spans="1:10" ht="20" customHeight="1">
+    <row r="10" spans="1:9" ht="20" customHeight="1">
       <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
+      <c r="B10" s="4"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -600,7 +583,7 @@
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
     </row>
-    <row r="11" spans="1:10" ht="20" customHeight="1">
+    <row r="11" spans="1:9" ht="20" customHeight="1">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -611,7 +594,7 @@
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
     </row>
-    <row r="12" spans="1:10" ht="20" customHeight="1">
+    <row r="12" spans="1:9" ht="20" customHeight="1">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -622,9 +605,9 @@
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
     </row>
-    <row r="13" spans="1:10" ht="20" customHeight="1">
+    <row r="13" spans="1:9" ht="20" customHeight="1">
       <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
+      <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
@@ -633,7 +616,7 @@
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:10" ht="20" customHeight="1">
+    <row r="14" spans="1:9" ht="20" customHeight="1">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -644,7 +627,7 @@
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
     </row>
-    <row r="15" spans="1:10" ht="20" customHeight="1">
+    <row r="15" spans="1:9" ht="20" customHeight="1">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -655,7 +638,7 @@
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
     </row>
-    <row r="16" spans="1:10" ht="20" customHeight="1">
+    <row r="16" spans="1:9" ht="20" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -1611,39 +1594,6 @@
       <c r="G102" s="3"/>
       <c r="H102" s="3"/>
       <c r="I102" s="3"/>
-    </row>
-    <row r="103" spans="1:9" ht="20" customHeight="1">
-      <c r="A103" s="3"/>
-      <c r="B103" s="3"/>
-      <c r="C103" s="3"/>
-      <c r="D103" s="3"/>
-      <c r="E103" s="3"/>
-      <c r="F103" s="3"/>
-      <c r="G103" s="3"/>
-      <c r="H103" s="3"/>
-      <c r="I103" s="3"/>
-    </row>
-    <row r="104" spans="1:9" ht="20" customHeight="1">
-      <c r="A104" s="3"/>
-      <c r="B104" s="3"/>
-      <c r="C104" s="3"/>
-      <c r="D104" s="3"/>
-      <c r="E104" s="3"/>
-      <c r="F104" s="3"/>
-      <c r="G104" s="3"/>
-      <c r="H104" s="3"/>
-      <c r="I104" s="3"/>
-    </row>
-    <row r="105" spans="1:9" ht="20" customHeight="1">
-      <c r="A105" s="3"/>
-      <c r="B105" s="3"/>
-      <c r="C105" s="3"/>
-      <c r="D105" s="3"/>
-      <c r="E105" s="3"/>
-      <c r="F105" s="3"/>
-      <c r="G105" s="3"/>
-      <c r="H105" s="3"/>
-      <c r="I105" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1663,10 +1613,10 @@
   <sheetData>
     <row r="1" spans="1:9" ht="35.25" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1685,47 +1635,47 @@
         <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="20" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="20" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="20" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="20" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="20" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="20" customHeight="1">
@@ -1734,66 +1684,66 @@
     </row>
     <row r="10" spans="1:9" ht="20" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="20" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="20" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="20" customHeight="1">
       <c r="A13" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="20" customHeight="1">
       <c r="A14" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="20" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="20" customHeight="1">
       <c r="A16" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="20" customHeight="1">
       <c r="A17" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="20" customHeight="1">
@@ -1802,66 +1752,66 @@
     </row>
     <row r="19" spans="1:2" ht="20" customHeight="1">
       <c r="A19" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="20" customHeight="1">
       <c r="A20" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="20" customHeight="1">
       <c r="A21" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="20" customHeight="1">
       <c r="A22" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="20" customHeight="1">
       <c r="A23" s="3" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="20" customHeight="1">
       <c r="A24" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="20" customHeight="1">
       <c r="A25" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="20" customHeight="1">
       <c r="A26" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update DeepSeek collector parsing
</commit_message>
<xml_diff>
--- a/questions.backup-before-more-questions.xlsx
+++ b/questions.backup-before-more-questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pan/Documents/思阳/Automatic-screenshot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20621BF0-2647-DF45-87E3-622B31F346B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61C1C06F-E91D-7C46-AD07-4D7A58ACF6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-2060" yWindow="-22000" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -173,22 +173,22 @@
     <t>Set status = success or failed with remark.</t>
   </si>
   <si>
-    <t>Q031</t>
-  </si>
-  <si>
-    <t>推荐一下家用烘干机怎么选</t>
-  </si>
-  <si>
-    <t>Q032</t>
-  </si>
-  <si>
-    <t>推荐几款扫拖一体机器人</t>
-  </si>
-  <si>
-    <t>Q033</t>
-  </si>
-  <si>
-    <t>推荐一下适合家用的空气净化器</t>
+    <t>Q020</t>
+  </si>
+  <si>
+    <t>推荐几款适合新手的厨刀套装</t>
+  </si>
+  <si>
+    <t>Q021</t>
+  </si>
+  <si>
+    <t>推荐一下家用咖啡机</t>
+  </si>
+  <si>
+    <t>Q022</t>
+  </si>
+  <si>
+    <t>推荐几款小型制冰机</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Add multi-session DeepSeek collection support
</commit_message>
<xml_diff>
--- a/questions.backup-before-more-questions.xlsx
+++ b/questions.backup-before-more-questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pan/Documents/思阳/Automatic-screenshot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61C1C06F-E91D-7C46-AD07-4D7A58ACF6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FBFEB81-E210-D545-AE23-6D0D4222EC9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-2060" yWindow="-22000" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
   <si>
     <t>id</t>
   </si>
@@ -173,22 +173,40 @@
     <t>Set status = success or failed with remark.</t>
   </si>
   <si>
-    <t>Q020</t>
-  </si>
-  <si>
-    <t>推荐几款适合新手的厨刀套装</t>
-  </si>
-  <si>
-    <t>Q021</t>
-  </si>
-  <si>
-    <t>推荐一下家用咖啡机</t>
-  </si>
-  <si>
-    <t>Q022</t>
-  </si>
-  <si>
-    <t>推荐几款小型制冰机</t>
+    <t>Q006</t>
+  </si>
+  <si>
+    <t>推荐几款好用的空气炸锅</t>
+  </si>
+  <si>
+    <t>Q007</t>
+  </si>
+  <si>
+    <t>推荐一下适合家庭用的净水器</t>
+  </si>
+  <si>
+    <t>Q008</t>
+  </si>
+  <si>
+    <t>推荐几款厨房用垃圾处理器</t>
+  </si>
+  <si>
+    <t>Q009</t>
+  </si>
+  <si>
+    <t>推荐一下家用智能油烟机</t>
+  </si>
+  <si>
+    <t>Q010</t>
+  </si>
+  <si>
+    <t>推荐几款好清洁的燃气灶</t>
+  </si>
+  <si>
+    <t>Q011</t>
+  </si>
+  <si>
+    <t>推荐一下嵌入式冰箱怎么选</t>
   </si>
 </sst>
 </file>
@@ -517,34 +535,64 @@
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
     </row>
-    <row r="5" spans="1:9" ht="20" customHeight="1">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
+    <row r="5" spans="1:9" ht="26.75" customHeight="1">
+      <c r="A5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
     </row>
-    <row r="6" spans="1:9" ht="20" customHeight="1">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
+    <row r="6" spans="1:9" ht="26.75" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="3">
+        <v>1</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
     </row>
-    <row r="7" spans="1:9" ht="20" customHeight="1">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
+    <row r="7" spans="1:9" ht="26.75" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>

</xml_diff>